<commit_message>
Allow processings of multiple crustal dip model branches
</commit_message>
<xml_diff>
--- a/data/branch_weight_data_v0-1.xlsx
+++ b/data/branch_weight_data_v0-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\McGrath\occ-coseismic\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57EF525B-C3E7-4D1D-A918-5858FCE1E18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C162FE-D9E6-4692-B90D-C0A60E7A23D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-105" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38055" yWindow="2940" windowWidth="32160" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="all sheets" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">crustal_weights_4_2!$L$1:$L$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">crustal_weights_swing_dip!$A$1:$G$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="314">
   <si>
     <t>N</t>
   </si>
@@ -946,37 +947,46 @@
     <t>NZSHM22_InversionSolution-QXV0b21hdGlvblRhc2s6NjkzMjUwOQ==</t>
   </si>
   <si>
-    <t>_c_BLDL</t>
-  </si>
-  <si>
-    <t>_c_BLDH</t>
-  </si>
-  <si>
-    <t>_c_BLDP</t>
-  </si>
-  <si>
-    <t>_c_BMDH</t>
-  </si>
-  <si>
-    <t>_c_BMDL</t>
-  </si>
-  <si>
-    <t>_c_BMDP</t>
-  </si>
-  <si>
-    <t>_c_BHDH</t>
-  </si>
-  <si>
-    <t>_c_BHDL</t>
-  </si>
-  <si>
-    <t>_c_BHDP</t>
-  </si>
-  <si>
     <t>dip_model</t>
   </si>
   <si>
     <t>dip_weight</t>
+  </si>
+  <si>
+    <t>n_td</t>
+  </si>
+  <si>
+    <t>n_def</t>
+  </si>
+  <si>
+    <t>n_dips</t>
+  </si>
+  <si>
+    <t>_c_LOIP</t>
+  </si>
+  <si>
+    <t>_c_MOIP</t>
+  </si>
+  <si>
+    <t>_c_HOIP</t>
+  </si>
+  <si>
+    <t>_c_LOIL</t>
+  </si>
+  <si>
+    <t>_c_MOIL</t>
+  </si>
+  <si>
+    <t>_c_HOIL</t>
+  </si>
+  <si>
+    <t>_c_LOIH</t>
+  </si>
+  <si>
+    <t>_c_MOIH</t>
+  </si>
+  <si>
+    <t>_c_HOIH</t>
   </si>
 </sst>
 </file>
@@ -4453,7 +4463,7 @@
         <v>0.505</v>
       </c>
       <c r="K3">
-        <f t="shared" ref="K2:K37" si="0">PRODUCT(G3:J3)</f>
+        <f t="shared" ref="K3:K37" si="0">PRODUCT(G3:J3)</f>
         <v>1.279367E-2</v>
       </c>
       <c r="L3">
@@ -6281,7 +6291,8 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCFFA5B5-D9A2-4366-B369-676754E8E9F5}">
-  <dimension ref="A1:T10"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:AB28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
@@ -6296,7 +6307,7 @@
     <col min="19" max="19" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6316,7 +6327,7 @@
         <v>251</v>
       </c>
       <c r="G1" t="s">
-        <v>309</v>
+        <v>300</v>
       </c>
       <c r="H1" t="s">
         <v>246</v>
@@ -6331,7 +6342,7 @@
         <v>248</v>
       </c>
       <c r="L1" t="s">
-        <v>310</v>
+        <v>301</v>
       </c>
       <c r="M1" t="s">
         <v>249</v>
@@ -6357,8 +6368,26 @@
       <c r="T1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="W1" t="s">
+        <v>303</v>
+      </c>
+      <c r="X1">
+        <v>1</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>302</v>
+      </c>
+      <c r="Z1">
+        <v>1</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>304</v>
+      </c>
+      <c r="AB1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2.7</v>
       </c>
@@ -6378,7 +6407,7 @@
         <v>250</v>
       </c>
       <c r="G2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="H2">
         <v>0.23899999999999999</v>
@@ -6393,31 +6422,31 @@
         <v>0.505</v>
       </c>
       <c r="L2">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="M2">
         <f>PRODUCT(H2:L2)</f>
-        <v>7.7697406250000003E-3</v>
+        <v>1.5539481250000001E-2</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="O2">
         <f>M2*N2</f>
-        <v>7.7697406250000003E-3</v>
+        <v>1.5539481250000004E-2</v>
       </c>
       <c r="P2">
-        <f>0.25*O2/SUM(O$2:O$10)</f>
-        <v>1.9850881036539765E-2</v>
+        <f>(1/($X$1*$Z$1*$AB$1)*O2/SUM($O$2:$O$10))</f>
+        <v>7.6621683374330285E-2</v>
       </c>
       <c r="Q2" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="S2" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2.7</v>
       </c>
@@ -6428,7 +6457,7 @@
         <v>4.2</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0.66</v>
       </c>
       <c r="E3" t="s">
         <v>131</v>
@@ -6437,13 +6466,13 @@
         <v>250</v>
       </c>
       <c r="G3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H3">
         <v>0.23899999999999999</v>
       </c>
       <c r="I3">
-        <v>0.51500000000000001</v>
+        <v>0.21199999999999999</v>
       </c>
       <c r="J3">
         <v>0.5</v>
@@ -6452,31 +6481,28 @@
         <v>0.505</v>
       </c>
       <c r="L3">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="M3">
-        <f>PRODUCT(H3:L3)</f>
-        <v>7.7697406250000003E-3</v>
+        <f t="shared" ref="M3:M10" si="0">PRODUCT(H3:L3)</f>
+        <v>6.396835E-3</v>
       </c>
       <c r="N3">
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="O3">
         <f>M3*N3</f>
-        <v>7.7697406250000003E-3</v>
+        <v>6.3968350000000018E-3</v>
       </c>
       <c r="P3">
-        <f t="shared" ref="P3:P10" si="0">0.25*O3/SUM(O$2:O$10)</f>
-        <v>1.9850881036539765E-2</v>
+        <f t="shared" ref="P3:P10" si="1">(1/($X$1*$Z$1*$AB$1)*O3/SUM($O$2:$O$10))</f>
+        <v>3.1541353156034985E-2</v>
       </c>
       <c r="Q3" t="s">
-        <v>300</v>
-      </c>
-      <c r="S3" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2.7</v>
       </c>
@@ -6487,7 +6513,7 @@
         <v>4.2</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>1.41</v>
       </c>
       <c r="E4" t="s">
         <v>131</v>
@@ -6502,7 +6528,7 @@
         <v>0.23899999999999999</v>
       </c>
       <c r="I4">
-        <v>0.51500000000000001</v>
+        <v>0.27300000000000002</v>
       </c>
       <c r="J4">
         <v>0.5</v>
@@ -6514,28 +6540,25 @@
         <v>0.5</v>
       </c>
       <c r="M4">
-        <f>PRODUCT(H4:L4)</f>
-        <v>1.5539481250000001E-2</v>
+        <f t="shared" si="0"/>
+        <v>8.2374337500000002E-3</v>
       </c>
       <c r="N4">
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="O4">
-        <f>M4*N4</f>
-        <v>1.5539481250000001E-2</v>
+        <f t="shared" ref="O4:O10" si="2">M4*N4</f>
+        <v>8.2374337500000019E-3</v>
       </c>
       <c r="P4">
-        <f t="shared" si="0"/>
-        <v>3.970176207307953E-2</v>
+        <f t="shared" si="1"/>
+        <v>4.0616931186780905E-2</v>
       </c>
       <c r="Q4" t="s">
-        <v>302</v>
-      </c>
-      <c r="S4" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3.4</v>
       </c>
@@ -6555,7 +6578,7 @@
         <v>250</v>
       </c>
       <c r="G5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="H5">
         <v>0.53600000000000003</v>
@@ -6570,31 +6593,31 @@
         <v>0.505</v>
       </c>
       <c r="L5">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="M5">
-        <f>PRODUCT(H5:L5)</f>
-        <v>1.7425025E-2</v>
+        <f t="shared" si="0"/>
+        <v>3.485005E-2</v>
       </c>
       <c r="N5">
-        <v>0.748107262752845</v>
+        <v>0.51113125501653078</v>
       </c>
       <c r="O5">
-        <f t="shared" ref="O5" si="1">M5*N5</f>
-        <v>1.3035787756149893E-2</v>
+        <f>M5*N5</f>
+        <v>1.7812949793888849E-2</v>
       </c>
       <c r="P5">
-        <f t="shared" si="0"/>
-        <v>3.3305085002745913E-2</v>
+        <f t="shared" si="1"/>
+        <v>8.7831644899355493E-2</v>
       </c>
       <c r="Q5" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="S5" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3.4</v>
       </c>
@@ -6605,7 +6628,7 @@
         <v>4.2</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0.66</v>
       </c>
       <c r="E6" t="s">
         <v>131</v>
@@ -6614,13 +6637,13 @@
         <v>250</v>
       </c>
       <c r="G6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H6">
         <v>0.53600000000000003</v>
       </c>
       <c r="I6">
-        <v>0.51500000000000001</v>
+        <v>0.21199999999999999</v>
       </c>
       <c r="J6">
         <v>0.5</v>
@@ -6629,31 +6652,28 @@
         <v>0.505</v>
       </c>
       <c r="L6">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="M6">
-        <f>PRODUCT(H6:L6)</f>
-        <v>1.7425025E-2</v>
+        <f t="shared" si="0"/>
+        <v>1.4346039999999999E-2</v>
       </c>
       <c r="N6">
-        <v>0.748107262752845</v>
+        <v>0.51113125501653078</v>
       </c>
       <c r="O6">
-        <f t="shared" ref="O6" si="2">M6*N6</f>
-        <v>1.3035787756149893E-2</v>
+        <f t="shared" si="2"/>
+        <v>7.3327094297173509E-3</v>
       </c>
       <c r="P6">
-        <f t="shared" si="0"/>
-        <v>3.3305085002745913E-2</v>
+        <f t="shared" si="1"/>
+        <v>3.6155939259540512E-2</v>
       </c>
       <c r="Q6" t="s">
-        <v>304</v>
-      </c>
-      <c r="S6" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3.4</v>
       </c>
@@ -6664,7 +6684,7 @@
         <v>4.2</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>1.41</v>
       </c>
       <c r="E7" t="s">
         <v>131</v>
@@ -6679,7 +6699,7 @@
         <v>0.53600000000000003</v>
       </c>
       <c r="I7">
-        <v>0.51500000000000001</v>
+        <v>0.27300000000000002</v>
       </c>
       <c r="J7">
         <v>0.5</v>
@@ -6691,28 +6711,25 @@
         <v>0.5</v>
       </c>
       <c r="M7">
-        <f>PRODUCT(H7:L7)</f>
-        <v>3.485005E-2</v>
+        <f t="shared" si="0"/>
+        <v>1.8473910000000003E-2</v>
       </c>
       <c r="N7">
-        <v>0.748107262752845</v>
+        <v>0.51113125501653078</v>
       </c>
       <c r="O7">
-        <f t="shared" ref="O7:O10" si="3">M7*N7</f>
-        <v>2.6071575512299786E-2</v>
+        <f t="shared" si="2"/>
+        <v>9.4425928033624405E-3</v>
       </c>
       <c r="P7">
-        <f t="shared" si="0"/>
-        <v>6.6610170005491826E-2</v>
+        <f t="shared" si="1"/>
+        <v>4.6559299140823407E-2</v>
       </c>
       <c r="Q7" t="s">
-        <v>305</v>
-      </c>
-      <c r="S7" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4.5999999999999996</v>
       </c>
@@ -6732,7 +6749,7 @@
         <v>250</v>
       </c>
       <c r="G8" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="H8">
         <v>0.22500000000000001</v>
@@ -6747,31 +6764,31 @@
         <v>0.505</v>
       </c>
       <c r="L8">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="M8">
-        <f>PRODUCT(H8:L8)</f>
-        <v>7.3146093750000004E-3</v>
+        <f t="shared" si="0"/>
+        <v>1.4629218750000001E-2</v>
       </c>
       <c r="N8">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="O8">
-        <f t="shared" ref="O8" si="4">M8*N8</f>
-        <v>3.6573046875000002E-3</v>
+        <f t="shared" si="2"/>
+        <v>1.4629218750000002E-3</v>
       </c>
       <c r="P8">
-        <f t="shared" si="0"/>
-        <v>9.3440339607143239E-3</v>
+        <f t="shared" si="1"/>
+        <v>7.2133383929808836E-3</v>
       </c>
       <c r="Q8" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="S8" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>4.5999999999999996</v>
       </c>
@@ -6782,7 +6799,7 @@
         <v>4.2</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>0.66</v>
       </c>
       <c r="E9" t="s">
         <v>131</v>
@@ -6791,13 +6808,13 @@
         <v>250</v>
       </c>
       <c r="G9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H9">
         <v>0.22500000000000001</v>
       </c>
       <c r="I9">
-        <v>0.51500000000000001</v>
+        <v>0.21199999999999999</v>
       </c>
       <c r="J9">
         <v>0.5</v>
@@ -6806,31 +6823,28 @@
         <v>0.505</v>
       </c>
       <c r="L9">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="M9">
-        <f>PRODUCT(H9:L9)</f>
-        <v>7.3146093750000004E-3</v>
+        <f t="shared" si="0"/>
+        <v>6.0221249999999997E-3</v>
       </c>
       <c r="N9">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="O9">
-        <f t="shared" ref="O9" si="5">M9*N9</f>
-        <v>3.6573046875000002E-3</v>
+        <f t="shared" si="2"/>
+        <v>6.0221250000000004E-4</v>
       </c>
       <c r="P9">
-        <f t="shared" si="0"/>
-        <v>9.3440339607143239E-3</v>
+        <f t="shared" si="1"/>
+        <v>2.9693742510911595E-3</v>
       </c>
       <c r="Q9" t="s">
         <v>307</v>
       </c>
-      <c r="S9" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4.5999999999999996</v>
       </c>
@@ -6841,7 +6855,7 @@
         <v>4.2</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>1.41</v>
       </c>
       <c r="E10" t="s">
         <v>131</v>
@@ -6856,7 +6870,7 @@
         <v>0.22500000000000001</v>
       </c>
       <c r="I10">
-        <v>0.51500000000000001</v>
+        <v>0.27300000000000002</v>
       </c>
       <c r="J10">
         <v>0.5</v>
@@ -6868,28 +6882,1058 @@
         <v>0.5</v>
       </c>
       <c r="M10">
-        <f>PRODUCT(H10:L10)</f>
-        <v>1.4629218750000001E-2</v>
+        <f t="shared" si="0"/>
+        <v>7.7549062500000014E-3</v>
       </c>
       <c r="N10">
+        <v>0.1</v>
+      </c>
+      <c r="O10">
+        <f t="shared" si="2"/>
+        <v>7.754906250000002E-4</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="1"/>
+        <v>3.8237696723956919E-3</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2.7</v>
+      </c>
+      <c r="B11">
+        <v>0.82299999999999995</v>
+      </c>
+      <c r="C11">
+        <v>4.2</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>131</v>
+      </c>
+      <c r="F11" t="s">
+        <v>250</v>
+      </c>
+      <c r="G11" t="s">
+        <v>290</v>
+      </c>
+      <c r="H11">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="I11">
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="J11">
         <v>0.5</v>
       </c>
-      <c r="O10">
+      <c r="K11">
+        <v>0.505</v>
+      </c>
+      <c r="L11">
+        <v>0.25</v>
+      </c>
+      <c r="M11">
+        <f t="shared" ref="M11:M28" si="3">PRODUCT(H11:L11)</f>
+        <v>7.7697406250000003E-3</v>
+      </c>
+      <c r="N11">
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="O11">
+        <f>M11*N11</f>
+        <v>7.7697406250000021E-3</v>
+      </c>
+      <c r="P11">
+        <f>(1/($X$1*$Z$1*$AB$1)*O11/SUM($O$11:$O$19))</f>
+        <v>7.6621683374330285E-2</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>308</v>
+      </c>
+      <c r="S11" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2.7</v>
+      </c>
+      <c r="B12">
+        <v>0.82299999999999995</v>
+      </c>
+      <c r="C12">
+        <v>4.2</v>
+      </c>
+      <c r="D12">
+        <v>0.66</v>
+      </c>
+      <c r="E12" t="s">
+        <v>131</v>
+      </c>
+      <c r="F12" t="s">
+        <v>250</v>
+      </c>
+      <c r="G12" t="s">
+        <v>290</v>
+      </c>
+      <c r="H12">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="I12">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="J12">
+        <v>0.5</v>
+      </c>
+      <c r="K12">
+        <v>0.505</v>
+      </c>
+      <c r="L12">
+        <v>0.25</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="3"/>
+        <v>3.1984175E-3</v>
+      </c>
+      <c r="N12">
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="O12">
+        <f>M12*N12</f>
+        <v>3.1984175000000009E-3</v>
+      </c>
+      <c r="P12">
+        <f t="shared" ref="P12:P19" si="4">(1/($X$1*$Z$1*$AB$1)*O12/SUM($O$11:$O$19))</f>
+        <v>3.1541353156034985E-2</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2.7</v>
+      </c>
+      <c r="B13">
+        <v>0.82299999999999995</v>
+      </c>
+      <c r="C13">
+        <v>4.2</v>
+      </c>
+      <c r="D13">
+        <v>1.41</v>
+      </c>
+      <c r="E13" t="s">
+        <v>131</v>
+      </c>
+      <c r="F13" t="s">
+        <v>250</v>
+      </c>
+      <c r="G13" t="s">
+        <v>290</v>
+      </c>
+      <c r="H13">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="I13">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="J13">
+        <v>0.5</v>
+      </c>
+      <c r="K13">
+        <v>0.505</v>
+      </c>
+      <c r="L13">
+        <v>0.25</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="3"/>
+        <v>4.1187168750000001E-3</v>
+      </c>
+      <c r="N13">
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="O13">
+        <f t="shared" ref="O13" si="5">M13*N13</f>
+        <v>4.118716875000001E-3</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="4"/>
+        <v>4.0616931186780905E-2</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>3.4</v>
+      </c>
+      <c r="B14">
+        <v>0.95899999999999996</v>
+      </c>
+      <c r="C14">
+        <v>4.2</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>131</v>
+      </c>
+      <c r="F14" t="s">
+        <v>250</v>
+      </c>
+      <c r="G14" t="s">
+        <v>290</v>
+      </c>
+      <c r="H14">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="I14">
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="J14">
+        <v>0.5</v>
+      </c>
+      <c r="K14">
+        <v>0.505</v>
+      </c>
+      <c r="L14">
+        <v>0.25</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="3"/>
+        <v>1.7425025E-2</v>
+      </c>
+      <c r="N14">
+        <v>0.51113125501653078</v>
+      </c>
+      <c r="O14">
+        <f>M14*N14</f>
+        <v>8.9064748969444243E-3</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="4"/>
+        <v>8.7831644899355493E-2</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>309</v>
+      </c>
+      <c r="S14" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>3.4</v>
+      </c>
+      <c r="B15">
+        <v>0.95899999999999996</v>
+      </c>
+      <c r="C15">
+        <v>4.2</v>
+      </c>
+      <c r="D15">
+        <v>0.66</v>
+      </c>
+      <c r="E15" t="s">
+        <v>131</v>
+      </c>
+      <c r="F15" t="s">
+        <v>250</v>
+      </c>
+      <c r="G15" t="s">
+        <v>290</v>
+      </c>
+      <c r="H15">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="I15">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="J15">
+        <v>0.5</v>
+      </c>
+      <c r="K15">
+        <v>0.505</v>
+      </c>
+      <c r="L15">
+        <v>0.25</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="3"/>
+        <v>7.1730199999999996E-3</v>
+      </c>
+      <c r="N15">
+        <v>0.51113125501653078</v>
+      </c>
+      <c r="O15">
+        <f t="shared" ref="O15:O19" si="6">M15*N15</f>
+        <v>3.6663547148586754E-3</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="4"/>
+        <v>3.6155939259540512E-2</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>3.4</v>
+      </c>
+      <c r="B16">
+        <v>0.95899999999999996</v>
+      </c>
+      <c r="C16">
+        <v>4.2</v>
+      </c>
+      <c r="D16">
+        <v>1.41</v>
+      </c>
+      <c r="E16" t="s">
+        <v>131</v>
+      </c>
+      <c r="F16" t="s">
+        <v>250</v>
+      </c>
+      <c r="G16" t="s">
+        <v>290</v>
+      </c>
+      <c r="H16">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="I16">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="J16">
+        <v>0.5</v>
+      </c>
+      <c r="K16">
+        <v>0.505</v>
+      </c>
+      <c r="L16">
+        <v>0.25</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="3"/>
+        <v>9.2369550000000016E-3</v>
+      </c>
+      <c r="N16">
+        <v>0.51113125501653078</v>
+      </c>
+      <c r="O16">
+        <f t="shared" si="6"/>
+        <v>4.7212964016812202E-3</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="4"/>
+        <v>4.6559299140823407E-2</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="B17">
+        <v>1.089</v>
+      </c>
+      <c r="C17">
+        <v>4.2</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
+        <v>131</v>
+      </c>
+      <c r="F17" t="s">
+        <v>250</v>
+      </c>
+      <c r="G17" t="s">
+        <v>290</v>
+      </c>
+      <c r="H17">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="I17">
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="J17">
+        <v>0.5</v>
+      </c>
+      <c r="K17">
+        <v>0.505</v>
+      </c>
+      <c r="L17">
+        <v>0.25</v>
+      </c>
+      <c r="M17">
         <f t="shared" si="3"/>
         <v>7.3146093750000004E-3</v>
       </c>
-      <c r="P10">
-        <f t="shared" si="0"/>
-        <v>1.8688067921428648E-2</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>308</v>
-      </c>
-      <c r="S10" t="s">
-        <v>299</v>
+      <c r="N17">
+        <v>0.1</v>
+      </c>
+      <c r="O17">
+        <f t="shared" si="6"/>
+        <v>7.3146093750000012E-4</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="4"/>
+        <v>7.2133383929808836E-3</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>310</v>
+      </c>
+      <c r="S17" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="B18">
+        <v>1.089</v>
+      </c>
+      <c r="C18">
+        <v>4.2</v>
+      </c>
+      <c r="D18">
+        <v>0.66</v>
+      </c>
+      <c r="E18" t="s">
+        <v>131</v>
+      </c>
+      <c r="F18" t="s">
+        <v>250</v>
+      </c>
+      <c r="G18" t="s">
+        <v>290</v>
+      </c>
+      <c r="H18">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="I18">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="J18">
+        <v>0.5</v>
+      </c>
+      <c r="K18">
+        <v>0.505</v>
+      </c>
+      <c r="L18">
+        <v>0.25</v>
+      </c>
+      <c r="M18">
+        <f t="shared" si="3"/>
+        <v>3.0110624999999999E-3</v>
+      </c>
+      <c r="N18">
+        <v>0.1</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="6"/>
+        <v>3.0110625000000002E-4</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="4"/>
+        <v>2.9693742510911595E-3</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="B19">
+        <v>1.089</v>
+      </c>
+      <c r="C19">
+        <v>4.2</v>
+      </c>
+      <c r="D19">
+        <v>1.41</v>
+      </c>
+      <c r="E19" t="s">
+        <v>131</v>
+      </c>
+      <c r="F19" t="s">
+        <v>250</v>
+      </c>
+      <c r="G19" t="s">
+        <v>290</v>
+      </c>
+      <c r="H19">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="I19">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="J19">
+        <v>0.5</v>
+      </c>
+      <c r="K19">
+        <v>0.505</v>
+      </c>
+      <c r="L19">
+        <v>0.25</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="3"/>
+        <v>3.8774531250000007E-3</v>
+      </c>
+      <c r="N19">
+        <v>0.1</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="6"/>
+        <v>3.877453125000001E-4</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="4"/>
+        <v>3.8237696723956919E-3</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>2.7</v>
+      </c>
+      <c r="B20">
+        <v>0.82299999999999995</v>
+      </c>
+      <c r="C20">
+        <v>4.2</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>131</v>
+      </c>
+      <c r="F20" t="s">
+        <v>250</v>
+      </c>
+      <c r="G20" t="s">
+        <v>289</v>
+      </c>
+      <c r="H20">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="I20">
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="J20">
+        <v>0.5</v>
+      </c>
+      <c r="K20">
+        <v>0.505</v>
+      </c>
+      <c r="L20">
+        <v>0.25</v>
+      </c>
+      <c r="M20">
+        <f t="shared" si="3"/>
+        <v>7.7697406250000003E-3</v>
+      </c>
+      <c r="N20">
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="O20">
+        <f t="shared" ref="O20:O28" si="7">M20*N20</f>
+        <v>7.7697406250000021E-3</v>
+      </c>
+      <c r="P20">
+        <f>(1/($X$1*$Z$1*$AB$1)*O20/SUM($O$20:$O$28))</f>
+        <v>7.6621683374330285E-2</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>311</v>
+      </c>
+      <c r="S20" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>2.7</v>
+      </c>
+      <c r="B21">
+        <v>0.82299999999999995</v>
+      </c>
+      <c r="C21">
+        <v>4.2</v>
+      </c>
+      <c r="D21">
+        <v>0.66</v>
+      </c>
+      <c r="E21" t="s">
+        <v>131</v>
+      </c>
+      <c r="F21" t="s">
+        <v>250</v>
+      </c>
+      <c r="G21" t="s">
+        <v>289</v>
+      </c>
+      <c r="H21">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="I21">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="J21">
+        <v>0.5</v>
+      </c>
+      <c r="K21">
+        <v>0.505</v>
+      </c>
+      <c r="L21">
+        <v>0.25</v>
+      </c>
+      <c r="M21">
+        <f t="shared" si="3"/>
+        <v>3.1984175E-3</v>
+      </c>
+      <c r="N21">
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="O21">
+        <f t="shared" si="7"/>
+        <v>3.1984175000000009E-3</v>
+      </c>
+      <c r="P21">
+        <f t="shared" ref="P21:P28" si="8">(1/($X$1*$Z$1*$AB$1)*O21/SUM($O$20:$O$28))</f>
+        <v>3.1541353156034985E-2</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>2.7</v>
+      </c>
+      <c r="B22">
+        <v>0.82299999999999995</v>
+      </c>
+      <c r="C22">
+        <v>4.2</v>
+      </c>
+      <c r="D22">
+        <v>1.41</v>
+      </c>
+      <c r="E22" t="s">
+        <v>131</v>
+      </c>
+      <c r="F22" t="s">
+        <v>250</v>
+      </c>
+      <c r="G22" t="s">
+        <v>289</v>
+      </c>
+      <c r="H22">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="I22">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="J22">
+        <v>0.5</v>
+      </c>
+      <c r="K22">
+        <v>0.505</v>
+      </c>
+      <c r="L22">
+        <v>0.25</v>
+      </c>
+      <c r="M22">
+        <f t="shared" si="3"/>
+        <v>4.1187168750000001E-3</v>
+      </c>
+      <c r="N22">
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="O22">
+        <f t="shared" si="7"/>
+        <v>4.118716875000001E-3</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="8"/>
+        <v>4.0616931186780905E-2</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>3.4</v>
+      </c>
+      <c r="B23">
+        <v>0.95899999999999996</v>
+      </c>
+      <c r="C23">
+        <v>4.2</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" t="s">
+        <v>131</v>
+      </c>
+      <c r="F23" t="s">
+        <v>250</v>
+      </c>
+      <c r="G23" t="s">
+        <v>289</v>
+      </c>
+      <c r="H23">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="I23">
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="J23">
+        <v>0.5</v>
+      </c>
+      <c r="K23">
+        <v>0.505</v>
+      </c>
+      <c r="L23">
+        <v>0.25</v>
+      </c>
+      <c r="M23">
+        <f t="shared" si="3"/>
+        <v>1.7425025E-2</v>
+      </c>
+      <c r="N23">
+        <v>0.51113125501653078</v>
+      </c>
+      <c r="O23">
+        <f t="shared" si="7"/>
+        <v>8.9064748969444243E-3</v>
+      </c>
+      <c r="P23">
+        <f t="shared" si="8"/>
+        <v>8.7831644899355493E-2</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>312</v>
+      </c>
+      <c r="S23" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>3.4</v>
+      </c>
+      <c r="B24">
+        <v>0.95899999999999996</v>
+      </c>
+      <c r="C24">
+        <v>4.2</v>
+      </c>
+      <c r="D24">
+        <v>0.66</v>
+      </c>
+      <c r="E24" t="s">
+        <v>131</v>
+      </c>
+      <c r="F24" t="s">
+        <v>250</v>
+      </c>
+      <c r="G24" t="s">
+        <v>289</v>
+      </c>
+      <c r="H24">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="I24">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="J24">
+        <v>0.5</v>
+      </c>
+      <c r="K24">
+        <v>0.505</v>
+      </c>
+      <c r="L24">
+        <v>0.25</v>
+      </c>
+      <c r="M24">
+        <f t="shared" si="3"/>
+        <v>7.1730199999999996E-3</v>
+      </c>
+      <c r="N24">
+        <v>0.51113125501653078</v>
+      </c>
+      <c r="O24">
+        <f t="shared" si="7"/>
+        <v>3.6663547148586754E-3</v>
+      </c>
+      <c r="P24">
+        <f t="shared" si="8"/>
+        <v>3.6155939259540512E-2</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>3.4</v>
+      </c>
+      <c r="B25">
+        <v>0.95899999999999996</v>
+      </c>
+      <c r="C25">
+        <v>4.2</v>
+      </c>
+      <c r="D25">
+        <v>1.41</v>
+      </c>
+      <c r="E25" t="s">
+        <v>131</v>
+      </c>
+      <c r="F25" t="s">
+        <v>250</v>
+      </c>
+      <c r="G25" t="s">
+        <v>289</v>
+      </c>
+      <c r="H25">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="I25">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="J25">
+        <v>0.5</v>
+      </c>
+      <c r="K25">
+        <v>0.505</v>
+      </c>
+      <c r="L25">
+        <v>0.25</v>
+      </c>
+      <c r="M25">
+        <f t="shared" si="3"/>
+        <v>9.2369550000000016E-3</v>
+      </c>
+      <c r="N25">
+        <v>0.51113125501653078</v>
+      </c>
+      <c r="O25">
+        <f t="shared" si="7"/>
+        <v>4.7212964016812202E-3</v>
+      </c>
+      <c r="P25">
+        <f t="shared" si="8"/>
+        <v>4.6559299140823407E-2</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="B26">
+        <v>1.089</v>
+      </c>
+      <c r="C26">
+        <v>4.2</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26" t="s">
+        <v>131</v>
+      </c>
+      <c r="F26" t="s">
+        <v>250</v>
+      </c>
+      <c r="G26" t="s">
+        <v>289</v>
+      </c>
+      <c r="H26">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="I26">
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="J26">
+        <v>0.5</v>
+      </c>
+      <c r="K26">
+        <v>0.505</v>
+      </c>
+      <c r="L26">
+        <v>0.25</v>
+      </c>
+      <c r="M26">
+        <f t="shared" si="3"/>
+        <v>7.3146093750000004E-3</v>
+      </c>
+      <c r="N26">
+        <v>0.1</v>
+      </c>
+      <c r="O26">
+        <f t="shared" si="7"/>
+        <v>7.3146093750000012E-4</v>
+      </c>
+      <c r="P26">
+        <f t="shared" si="8"/>
+        <v>7.2133383929808836E-3</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>313</v>
+      </c>
+      <c r="S26" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="B27">
+        <v>1.089</v>
+      </c>
+      <c r="C27">
+        <v>4.2</v>
+      </c>
+      <c r="D27">
+        <v>0.66</v>
+      </c>
+      <c r="E27" t="s">
+        <v>131</v>
+      </c>
+      <c r="F27" t="s">
+        <v>250</v>
+      </c>
+      <c r="G27" t="s">
+        <v>289</v>
+      </c>
+      <c r="H27">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="I27">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="J27">
+        <v>0.5</v>
+      </c>
+      <c r="K27">
+        <v>0.505</v>
+      </c>
+      <c r="L27">
+        <v>0.25</v>
+      </c>
+      <c r="M27">
+        <f t="shared" si="3"/>
+        <v>3.0110624999999999E-3</v>
+      </c>
+      <c r="N27">
+        <v>0.1</v>
+      </c>
+      <c r="O27">
+        <f t="shared" si="7"/>
+        <v>3.0110625000000002E-4</v>
+      </c>
+      <c r="P27">
+        <f t="shared" si="8"/>
+        <v>2.9693742510911595E-3</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="B28">
+        <v>1.089</v>
+      </c>
+      <c r="C28">
+        <v>4.2</v>
+      </c>
+      <c r="D28">
+        <v>1.41</v>
+      </c>
+      <c r="E28" t="s">
+        <v>131</v>
+      </c>
+      <c r="F28" t="s">
+        <v>250</v>
+      </c>
+      <c r="G28" t="s">
+        <v>289</v>
+      </c>
+      <c r="H28">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="I28">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="J28">
+        <v>0.5</v>
+      </c>
+      <c r="K28">
+        <v>0.505</v>
+      </c>
+      <c r="L28">
+        <v>0.25</v>
+      </c>
+      <c r="M28">
+        <f t="shared" si="3"/>
+        <v>3.8774531250000007E-3</v>
+      </c>
+      <c r="N28">
+        <v>0.1</v>
+      </c>
+      <c r="O28">
+        <f t="shared" si="7"/>
+        <v>3.877453125000001E-4</v>
+      </c>
+      <c r="P28">
+        <f t="shared" si="8"/>
+        <v>3.8237696723956919E-3</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>313</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G28" xr:uid="{BCFFA5B5-D9A2-4366-B369-676754E8E9F5}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <headerFooter>

</xml_diff>